<commit_message>
Smile Tustin: add criterion (d) image alt-text findings (12 rows), regenerate xlsx
Completes the full method: exact-match geographic keyword alts + wrong-topic
alts + one alt reused across 9 root-canal pages. 22 action items total.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018G4x2nGmsTqbufqtgwY9ey
</commit_message>
<xml_diff>
--- a/tustin_july_ranking_drop.xlsx
+++ b/tustin_july_ranking_drop.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Smile Tustin" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Smile Tustin'!$A$1:$I$119</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Smile Tustin'!$A$1:$I$111</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -98,7 +98,7 @@
   <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I119"/>
+  <dimension ref="A1:I111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -834,42 +834,42 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>blogs index page</t>
+          <t>porcelain-veneers page</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/blogs/</t>
+          <t>https://smiletustin.com/tustin-ca/porcelain-veneers/</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Add</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>Low</t>
+          <t>Change</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Missing main heading (H1)</t>
+          <t>Image alt text (wrong topic)</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>(No H1 on the page)</t>
+          <t>Invisalign treatment in Tustin, CA</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Add an H1: Dental Blog</t>
+          <t>Dentist placing porcelain veneers</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>The blog listing page has no main heading.</t>
+          <t>On the veneers page an image is labeled as Invisalign and written as a location search phrase, which is both wrong and unnatural.</t>
         </is>
       </c>
     </row>
@@ -881,42 +881,42 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>survey page</t>
+          <t>tustin-teeth-cleaning-appointment blog</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/survey/</t>
+          <t>https://smiletustin.com/tustin-teeth-cleaning-appointment/</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Add</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>Low</t>
+          <t>Change</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Missing main heading (H1)</t>
+          <t>Image alt text (wrong topic)</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>(No H1 on the page)</t>
+          <t>smile makeovers in tustin cosmetic dentist</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Add an H1: Patient Survey</t>
+          <t>Patient at a dental cleaning visit</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>The page has no main heading at all.</t>
+          <t>The image is labeled with stacked location keywords that do not match the page (which is about a teeth cleaning appointment).</t>
         </is>
       </c>
     </row>
@@ -928,12 +928,12 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>fluoride-treatments page</t>
+          <t>preventative-dentistry page</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/tustin-ca/fluoride-treatments/</t>
+          <t>https://smiletustin.com/tustin-ca/preventative-dentistry/</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -941,29 +941,29 @@
           <t>Change</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>Low</t>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Page title (stray characters)</t>
+          <t>Image alt text (wrong topic)</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Top Fluoride Treatments in Tustin, CA -</t>
+          <t>Periodontal Therapy in Tustin</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Fluoride Treatments in Tustin, CA</t>
+          <t>Preventive dental checkup</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>The title ends with a stray " -" that should be removed.</t>
+          <t>On the preventive page an image is labeled as periodontal therapy and written as a location search phrase.</t>
         </is>
       </c>
     </row>
@@ -975,462 +975,606 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>blogs index page</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>https://smiletustin.com/blogs/</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Add</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Missing main heading (H1)</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>(No H1 on the page)</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Add an H1: Dental Blog</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>The blog listing page has no main heading.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>survey page</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>https://smiletustin.com/survey/</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Add</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Missing main heading (H1)</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>(No H1 on the page)</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Add an H1: Patient Survey</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>The page has no main heading at all.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>fluoride-treatments page</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>https://smiletustin.com/tustin-ca/fluoride-treatments/</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Change</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Page title (stray characters)</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Top Fluoride Treatments in Tustin, CA -</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Fluoride Treatments in Tustin, CA</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>The title ends with a stray " -" that should be removed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
           <t>central-orange-county blog</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>https://smiletustin.com/central-orange-county-living-why-tustin-offers-the-best-of-both-worlds/</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>Change</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>Page title (missing separator)</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>Central Orange County Living: Why Tustin Offers the Best of Both Worlds Smile Tustin by Dr. Ezzy</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>Central Orange County Living: Why Tustin Offers the Best of Both Worlds | Smile Tustin by Dr. Ezzy</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>The brand name is stuck to the end of the title with no separator before it.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>smiletustin.com page</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>https://smiletustin.com/</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="E12" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F12" s="7" t="inlineStr"/>
-      <c r="G12" s="7" t="inlineStr"/>
-      <c r="H12" s="7" t="inlineStr"/>
-      <c r="I12" s="7" t="inlineStr">
-        <is>
-          <t>Home page - ranks #1-4 for the main dentist/implant searches; title and H1 match. Do not touch during the core update.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>tustin-ca page</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>https://smiletustin.com/tustin-ca/</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F13" s="7" t="inlineStr"/>
-      <c r="G13" s="7" t="inlineStr"/>
-      <c r="H13" s="7" t="inlineStr"/>
-      <c r="I13" s="7" t="inlineStr">
-        <is>
-          <t>Title and heading match the page topic; no change needed now. Keep.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>thank-you page</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="inlineStr">
-        <is>
-          <t>https://smiletustin.com/thank-you/</t>
-        </is>
-      </c>
-      <c r="D14" s="7" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="E14" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F14" s="7" t="inlineStr"/>
-      <c r="G14" s="7" t="inlineStr"/>
-      <c r="H14" s="7" t="inlineStr"/>
-      <c r="I14" s="7" t="inlineStr">
-        <is>
-          <t>Utility/support page; fine as-is. Keep.</t>
-        </is>
-      </c>
-    </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>14</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>patient-reviews page</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="inlineStr">
-        <is>
-          <t>https://smiletustin.com/patient-reviews/</t>
-        </is>
-      </c>
-      <c r="D15" s="7" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="E15" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F15" s="7" t="inlineStr"/>
-      <c r="G15" s="7" t="inlineStr"/>
-      <c r="H15" s="7" t="inlineStr"/>
-      <c r="I15" s="7" t="inlineStr">
-        <is>
-          <t>Utility/support page; fine as-is. Keep.</t>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>dental-inlays-and-onlays page</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>https://smiletustin.com/tustin-ca/dental-inlays-and-onlays/</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Change</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Image alt text</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Dental Inlays and Onlays in Tustin, CA</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Close-up of a dental inlay and onlay</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>The image description is written as a location search phrase instead of describing the picture.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>links page</t>
-        </is>
-      </c>
-      <c r="C16" s="7" t="inlineStr">
-        <is>
-          <t>https://smiletustin.com/links/</t>
-        </is>
-      </c>
-      <c r="D16" s="7" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="E16" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F16" s="7" t="inlineStr"/>
-      <c r="G16" s="7" t="inlineStr"/>
-      <c r="H16" s="7" t="inlineStr"/>
-      <c r="I16" s="7" t="inlineStr">
-        <is>
-          <t>Utility/support page; fine as-is. Keep.</t>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>family-dentistry page</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>https://smiletustin.com/tustin-ca/family-dentistry/</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Change</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Image alt text</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Family Dentistry in Tustin, CA</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Family at the dentist</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>The image description is written as a location search phrase instead of describing the picture.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>cerec-one-visit-dentistry page</t>
-        </is>
-      </c>
-      <c r="C17" s="7" t="inlineStr">
-        <is>
-          <t>https://smiletustin.com/cerec-one-visit-dentistry/</t>
-        </is>
-      </c>
-      <c r="D17" s="7" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="E17" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F17" s="7" t="inlineStr"/>
-      <c r="G17" s="7" t="inlineStr"/>
-      <c r="H17" s="7" t="inlineStr"/>
-      <c r="I17" s="7" t="inlineStr">
-        <is>
-          <t>Title and heading match the page topic; no change needed now. Keep.</t>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>dental-bridge page</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>https://smiletustin.com/tustin-ca/dental-bridge/</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Change</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Image alt text</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Dental Bridges in Tustin, CA</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Model of a dental bridge</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>The image description is written as a location search phrase instead of describing the picture.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>17</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>why-choose-us page</t>
-        </is>
-      </c>
-      <c r="C18" s="7" t="inlineStr">
-        <is>
-          <t>https://smiletustin.com/why-choose-us/</t>
-        </is>
-      </c>
-      <c r="D18" s="7" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="E18" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F18" s="7" t="inlineStr"/>
-      <c r="G18" s="7" t="inlineStr"/>
-      <c r="H18" s="7" t="inlineStr"/>
-      <c r="I18" s="7" t="inlineStr">
-        <is>
-          <t>Title and heading match the page topic; no change needed now. Keep.</t>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>iv-sedation page</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>https://smiletustin.com/tustin-ca/iv-sedation/</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Change</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Image alt text</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>IV Sedation Dentistry in Tustin, CA</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Patient relaxed under IV sedation</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>The image description is written as a location search phrase instead of describing the picture.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>18</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>3d-digital-dentistry page</t>
-        </is>
-      </c>
-      <c r="C19" s="7" t="inlineStr">
-        <is>
-          <t>https://smiletustin.com/3d-digital-dentistry/</t>
-        </is>
-      </c>
-      <c r="D19" s="7" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="E19" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F19" s="7" t="inlineStr"/>
-      <c r="G19" s="7" t="inlineStr"/>
-      <c r="H19" s="7" t="inlineStr"/>
-      <c r="I19" s="7" t="inlineStr">
-        <is>
-          <t>Title and heading match the page topic; no change needed now. Keep.</t>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>invisalign-clear-aligners page</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>https://smiletustin.com/tustin-ca/invisalign-clear-aligners/</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Change</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Image alt text</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Invisalign treatment in Tustin, CA</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Hand holding a clear Invisalign aligner</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>The image description is written as a location search phrase instead of describing the picture.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
-        <is>
-          <t>home-care page</t>
-        </is>
-      </c>
-      <c r="C20" s="7" t="inlineStr">
-        <is>
-          <t>https://smiletustin.com/home-care/</t>
-        </is>
-      </c>
-      <c r="D20" s="7" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="E20" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F20" s="7" t="inlineStr"/>
-      <c r="G20" s="7" t="inlineStr"/>
-      <c r="H20" s="7" t="inlineStr"/>
-      <c r="I20" s="7" t="inlineStr">
-        <is>
-          <t>Utility/support page; fine as-is. Keep.</t>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>dental-insurance-financing page</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>https://smiletustin.com/dental-insurance-financing/</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Change</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Image alt text</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Dental Insurance in Tustin</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Patient reviewing insurance and payment options</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>The image description is written as a location search phrase instead of describing the picture.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
-        <is>
-          <t>dr-kory-golchert-endodontist page</t>
-        </is>
-      </c>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>https://smiletustin.com/meet-our-dental-team/dr-kory-golchert-endodontist/</t>
-        </is>
-      </c>
-      <c r="D21" s="7" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="E21" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F21" s="7" t="inlineStr"/>
-      <c r="G21" s="7" t="inlineStr"/>
-      <c r="H21" s="7" t="inlineStr"/>
-      <c r="I21" s="7" t="inlineStr">
-        <is>
-          <t>Title and heading match the page topic; no change needed now. Keep.</t>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>new-year-new-smile blog</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>https://smiletustin.com/new-year-new-smile-find-your-local-dentist-in-tustin-for-2026/</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Change</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Image alt text</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>local dentist in Tustin</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Dentist welcoming a patient</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>The image description is written as a location search phrase instead of describing the picture.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>21</t>
         </is>
       </c>
-      <c r="B22" s="7" t="inlineStr">
-        <is>
-          <t>patients-first-visit page</t>
-        </is>
-      </c>
-      <c r="C22" s="7" t="inlineStr">
-        <is>
-          <t>https://smiletustin.com/patients-first-visit/</t>
-        </is>
-      </c>
-      <c r="D22" s="7" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="E22" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F22" s="7" t="inlineStr"/>
-      <c r="G22" s="7" t="inlineStr"/>
-      <c r="H22" s="7" t="inlineStr"/>
-      <c r="I22" s="7" t="inlineStr">
-        <is>
-          <t>Dedicated first-visit page; title and H1 match. Keep.</t>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>emergency-dental-care blog</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>https://smiletustin.com/emergency-dental-care-in-tustin-where-to-go-when-tooth-pain-strikes/</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Change</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Image alt text</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>emergency dental care in Tustin</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Person with a dental emergency</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>The image description is written as a location search phrase instead of describing the picture.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="inlineStr">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>22</t>
         </is>
       </c>
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>smile-gallery page</t>
-        </is>
-      </c>
-      <c r="C23" s="7" t="inlineStr">
-        <is>
-          <t>https://smiletustin.com/smile-gallery/</t>
-        </is>
-      </c>
-      <c r="D23" s="7" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F23" s="7" t="inlineStr"/>
-      <c r="G23" s="7" t="inlineStr"/>
-      <c r="H23" s="7" t="inlineStr"/>
-      <c r="I23" s="7" t="inlineStr">
-        <is>
-          <t>Utility/support page; fine as-is. Keep.</t>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>root canal pages (service + 8 blogs)</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>https://smiletustin.com/tustin-ca/root-canals/</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Change</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Image alt text (same alt reused on 9 pages)</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Root canal treatment in Tustin, CA  [same alt copied on: /tustin-ca/root-canals/, are-root-canals-painful, can-a-root-canal-procedure-save-your-tooth, factors-affect-root-canal-lifespan, dentist-for-emergency-root-canal, beyond-teeth-whitening-internal-bleaching, inside-smile-tustins-advanced-microscope-endodontics, the-truth-about-root-canals, am-i-a-candidate-for-root-canal]</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Give each image its own plain description (e.g. "Dentist performing a root canal"), without the city keyword</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>The identical location-keyword description is copied across nine root-canal pages instead of describing each image.</t>
         </is>
       </c>
     </row>
@@ -1442,12 +1586,12 @@
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>dr-zahra-hanieh-ezzy-tustin-dentist page</t>
+          <t>smiletustin.com page</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/meet-our-dental-team/dr-zahra-hanieh-ezzy-tustin-dentist/</t>
+          <t>https://smiletustin.com/</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
@@ -1465,7 +1609,7 @@
       <c r="H24" s="7" t="inlineStr"/>
       <c r="I24" s="7" t="inlineStr">
         <is>
-          <t>Title and heading match the page topic; no change needed now. Keep.</t>
+          <t>Home page - ranks #1-4 for the main dentist/implant searches; title and H1 match. Do not touch during the core update.</t>
         </is>
       </c>
     </row>
@@ -1477,12 +1621,12 @@
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>about-us page</t>
+          <t>tustin-ca page</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/about-us/</t>
+          <t>https://smiletustin.com/tustin-ca/</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
@@ -1512,12 +1656,12 @@
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>video-testimonials page</t>
+          <t>thank-you page</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/video-testimonials/</t>
+          <t>https://smiletustin.com/thank-you/</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
@@ -1547,12 +1691,12 @@
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>dental-videos page</t>
+          <t>patient-reviews page</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/dental-videos/</t>
+          <t>https://smiletustin.com/patient-reviews/</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
@@ -1582,12 +1726,12 @@
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>feedback page</t>
+          <t>links page</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/feedback/</t>
+          <t>https://smiletustin.com/links/</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
@@ -1617,12 +1761,12 @@
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>accessibility-statement page</t>
+          <t>cerec-one-visit-dentistry page</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/accessibility-statement/</t>
+          <t>https://smiletustin.com/cerec-one-visit-dentistry/</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
@@ -1640,7 +1784,7 @@
       <c r="H29" s="7" t="inlineStr"/>
       <c r="I29" s="7" t="inlineStr">
         <is>
-          <t>Legal/utility page; fine as-is. Keep.</t>
+          <t>Title and heading match the page topic; no change needed now. Keep.</t>
         </is>
       </c>
     </row>
@@ -1652,12 +1796,12 @@
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>privacy-policy page</t>
+          <t>why-choose-us page</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/privacy-policy/</t>
+          <t>https://smiletustin.com/why-choose-us/</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
@@ -1675,7 +1819,7 @@
       <c r="H30" s="7" t="inlineStr"/>
       <c r="I30" s="7" t="inlineStr">
         <is>
-          <t>Legal/utility page; fine as-is. Keep.</t>
+          <t>Title and heading match the page topic; no change needed now. Keep.</t>
         </is>
       </c>
     </row>
@@ -1687,12 +1831,12 @@
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>dentist-appointment page</t>
+          <t>3d-digital-dentistry page</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/dentist-appointment/</t>
+          <t>https://smiletustin.com/3d-digital-dentistry/</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
@@ -1722,12 +1866,12 @@
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>treatment-lanap page</t>
+          <t>home-care page</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/tustin-ca/treatment-lanap/</t>
+          <t>https://smiletustin.com/home-care/</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
@@ -1745,7 +1889,7 @@
       <c r="H32" s="7" t="inlineStr"/>
       <c r="I32" s="7" t="inlineStr">
         <is>
-          <t>Title and heading match the page topic; no change needed now. Keep.</t>
+          <t>Utility/support page; fine as-is. Keep.</t>
         </is>
       </c>
     </row>
@@ -1757,12 +1901,12 @@
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>dental-services page</t>
+          <t>dr-kory-golchert-endodontist page</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/dental-services/</t>
+          <t>https://smiletustin.com/meet-our-dental-team/dr-kory-golchert-endodontist/</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
@@ -1792,12 +1936,12 @@
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>dental-technology page</t>
+          <t>patients-first-visit page</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/dental-technology/</t>
+          <t>https://smiletustin.com/patients-first-visit/</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
@@ -1815,7 +1959,7 @@
       <c r="H34" s="7" t="inlineStr"/>
       <c r="I34" s="7" t="inlineStr">
         <is>
-          <t>Title and heading match the page topic; no change needed now. Keep.</t>
+          <t>Dedicated first-visit page; title and H1 match. Keep.</t>
         </is>
       </c>
     </row>
@@ -1827,12 +1971,12 @@
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>dental-insurance-financing page</t>
+          <t>smile-gallery page</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/dental-insurance-financing/</t>
+          <t>https://smiletustin.com/smile-gallery/</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
@@ -1850,7 +1994,7 @@
       <c r="H35" s="7" t="inlineStr"/>
       <c r="I35" s="7" t="inlineStr">
         <is>
-          <t>Title and heading match the page topic; no change needed now. Keep.</t>
+          <t>Utility/support page; fine as-is. Keep.</t>
         </is>
       </c>
     </row>
@@ -1862,12 +2006,12 @@
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>meet-our-dental-team page</t>
+          <t>dr-zahra-hanieh-ezzy-tustin-dentist page</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/meet-our-dental-team/</t>
+          <t>https://smiletustin.com/meet-our-dental-team/dr-zahra-hanieh-ezzy-tustin-dentist/</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
@@ -1897,12 +2041,12 @@
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>sleep-support-devices-snore-guard page</t>
+          <t>about-us page</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/tustin-ca/sleep-support-devices-snore-guard/</t>
+          <t>https://smiletustin.com/about-us/</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
@@ -1932,12 +2076,12 @@
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>prp-and-prf page</t>
+          <t>video-testimonials page</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/tustin-ca/prp-and-prf/</t>
+          <t>https://smiletustin.com/video-testimonials/</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
@@ -1955,7 +2099,7 @@
       <c r="H38" s="7" t="inlineStr"/>
       <c r="I38" s="7" t="inlineStr">
         <is>
-          <t>Title and heading match the page topic; no change needed now. Keep.</t>
+          <t>Utility/support page; fine as-is. Keep.</t>
         </is>
       </c>
     </row>
@@ -1967,12 +2111,12 @@
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>tmj-treatment page</t>
+          <t>dental-videos page</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/tustin-ca/tmj-treatment/</t>
+          <t>https://smiletustin.com/dental-videos/</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
@@ -1990,7 +2134,7 @@
       <c r="H39" s="7" t="inlineStr"/>
       <c r="I39" s="7" t="inlineStr">
         <is>
-          <t>Title and heading match the page topic; no change needed now. Keep.</t>
+          <t>Utility/support page; fine as-is. Keep.</t>
         </is>
       </c>
     </row>
@@ -2002,12 +2146,12 @@
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>bone-grafting page</t>
+          <t>feedback page</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/tustin-ca/bone-grafting/</t>
+          <t>https://smiletustin.com/feedback/</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
@@ -2025,7 +2169,7 @@
       <c r="H40" s="7" t="inlineStr"/>
       <c r="I40" s="7" t="inlineStr">
         <is>
-          <t>Title and heading match the page topic; no change needed now. Keep.</t>
+          <t>Utility/support page; fine as-is. Keep.</t>
         </is>
       </c>
     </row>
@@ -2037,12 +2181,12 @@
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>implant-supported-dentures page</t>
+          <t>accessibility-statement page</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/tustin-ca/implant-supported-dentures/</t>
+          <t>https://smiletustin.com/accessibility-statement/</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
@@ -2060,7 +2204,7 @@
       <c r="H41" s="7" t="inlineStr"/>
       <c r="I41" s="7" t="inlineStr">
         <is>
-          <t>Title and heading match the page topic; no change needed now. Keep.</t>
+          <t>Legal/utility page; fine as-is. Keep.</t>
         </is>
       </c>
     </row>
@@ -2072,12 +2216,12 @@
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>iv-sedation page</t>
+          <t>privacy-policy page</t>
         </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/tustin-ca/iv-sedation/</t>
+          <t>https://smiletustin.com/privacy-policy/</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
@@ -2095,7 +2239,7 @@
       <c r="H42" s="7" t="inlineStr"/>
       <c r="I42" s="7" t="inlineStr">
         <is>
-          <t>Title and heading match the page topic; no change needed now. Keep.</t>
+          <t>Legal/utility page; fine as-is. Keep.</t>
         </is>
       </c>
     </row>
@@ -2107,12 +2251,12 @@
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>internal-bleaching page</t>
+          <t>dentist-appointment page</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/tustin-ca/internal-bleaching/</t>
+          <t>https://smiletustin.com/dentist-appointment/</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
@@ -2130,7 +2274,7 @@
       <c r="H43" s="7" t="inlineStr"/>
       <c r="I43" s="7" t="inlineStr">
         <is>
-          <t>Main internal-bleaching page - the duplicate is pointed here. Keep.</t>
+          <t>Title and heading match the page topic; no change needed now. Keep.</t>
         </is>
       </c>
     </row>
@@ -2142,12 +2286,12 @@
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>preventative-dentistry page</t>
+          <t>treatment-lanap page</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/tustin-ca/preventative-dentistry/</t>
+          <t>https://smiletustin.com/tustin-ca/treatment-lanap/</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
@@ -2177,12 +2321,12 @@
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>cosmetic-dentistry page</t>
+          <t>dental-services page</t>
         </is>
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/tustin-ca/cosmetic-dentistry/</t>
+          <t>https://smiletustin.com/dental-services/</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
@@ -2212,12 +2356,12 @@
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>restorative-dentistry page</t>
+          <t>dental-technology page</t>
         </is>
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/tustin-ca/restorative-dentistry/</t>
+          <t>https://smiletustin.com/dental-technology/</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
@@ -2247,12 +2391,12 @@
       </c>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>dental-fillings page</t>
+          <t>meet-our-dental-team page</t>
         </is>
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/tustin-ca/dental-fillings/</t>
+          <t>https://smiletustin.com/meet-our-dental-team/</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr">
@@ -2270,7 +2414,7 @@
       <c r="H47" s="7" t="inlineStr"/>
       <c r="I47" s="7" t="inlineStr">
         <is>
-          <t>Main dental-fillings page - the duplicate is pointed here. Keep.</t>
+          <t>Title and heading match the page topic; no change needed now. Keep.</t>
         </is>
       </c>
     </row>
@@ -2282,12 +2426,12 @@
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>periodontal-care page</t>
+          <t>sleep-support-devices-snore-guard page</t>
         </is>
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/tustin-ca/periodontal-care/</t>
+          <t>https://smiletustin.com/tustin-ca/sleep-support-devices-snore-guard/</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
@@ -2317,12 +2461,12 @@
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>mouthguards page</t>
+          <t>prp-and-prf page</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/tustin-ca/mouthguards/</t>
+          <t>https://smiletustin.com/tustin-ca/prp-and-prf/</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
@@ -2352,12 +2496,12 @@
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>dental-inlays-and-onlays page</t>
+          <t>tmj-treatment page</t>
         </is>
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/tustin-ca/dental-inlays-and-onlays/</t>
+          <t>https://smiletustin.com/tustin-ca/tmj-treatment/</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
@@ -2387,12 +2531,12 @@
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>dental-exams page</t>
+          <t>bone-grafting page</t>
         </is>
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/tustin-ca/dental-exams/</t>
+          <t>https://smiletustin.com/tustin-ca/bone-grafting/</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
@@ -2422,12 +2566,12 @@
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>porcelain-veneers page</t>
+          <t>implant-supported-dentures page</t>
         </is>
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/tustin-ca/porcelain-veneers/</t>
+          <t>https://smiletustin.com/tustin-ca/implant-supported-dentures/</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
@@ -2457,12 +2601,12 @@
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>family-dentistry page</t>
+          <t>internal-bleaching page</t>
         </is>
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/tustin-ca/family-dentistry/</t>
+          <t>https://smiletustin.com/tustin-ca/internal-bleaching/</t>
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr">
@@ -2480,7 +2624,7 @@
       <c r="H53" s="7" t="inlineStr"/>
       <c r="I53" s="7" t="inlineStr">
         <is>
-          <t>Title and heading match the page topic; no change needed now. Keep.</t>
+          <t>Main internal-bleaching page - the duplicate is pointed here. Keep.</t>
         </is>
       </c>
     </row>
@@ -2492,12 +2636,12 @@
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>wisdom-teeth-removal page</t>
+          <t>cosmetic-dentistry page</t>
         </is>
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/tustin-ca/wisdom-teeth-removal/</t>
+          <t>https://smiletustin.com/tustin-ca/cosmetic-dentistry/</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
@@ -2527,12 +2671,12 @@
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>teeth-cleaning page</t>
+          <t>restorative-dentistry page</t>
         </is>
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/tustin-ca/teeth-cleaning/</t>
+          <t>https://smiletustin.com/tustin-ca/restorative-dentistry/</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
@@ -2562,12 +2706,12 @@
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>dental-bridge page</t>
+          <t>dental-fillings page</t>
         </is>
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/tustin-ca/dental-bridge/</t>
+          <t>https://smiletustin.com/tustin-ca/dental-fillings/</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
@@ -2585,7 +2729,7 @@
       <c r="H56" s="7" t="inlineStr"/>
       <c r="I56" s="7" t="inlineStr">
         <is>
-          <t>Title and heading match the page topic; no change needed now. Keep.</t>
+          <t>Main dental-fillings page - the duplicate is pointed here. Keep.</t>
         </is>
       </c>
     </row>
@@ -2597,12 +2741,12 @@
       </c>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>all-on-4-dental-implants page</t>
+          <t>periodontal-care page</t>
         </is>
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/tustin-ca/all-on-4-dental-implants/</t>
+          <t>https://smiletustin.com/tustin-ca/periodontal-care/</t>
         </is>
       </c>
       <c r="D57" s="7" t="inlineStr">
@@ -2632,12 +2776,12 @@
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>oral-surgery page</t>
+          <t>mouthguards page</t>
         </is>
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/tustin-ca/oral-surgery/</t>
+          <t>https://smiletustin.com/tustin-ca/mouthguards/</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
@@ -2667,12 +2811,12 @@
       </c>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>dentures-and-partial-dentures page</t>
+          <t>dental-exams page</t>
         </is>
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/tustin-ca/dentures-and-partial-dentures/</t>
+          <t>https://smiletustin.com/tustin-ca/dental-exams/</t>
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr">
@@ -2690,7 +2834,7 @@
       <c r="H59" s="7" t="inlineStr"/>
       <c r="I59" s="7" t="inlineStr">
         <is>
-          <t>Best result for "dentures tustin" (#1). Do not touch.</t>
+          <t>Title and heading match the page topic; no change needed now. Keep.</t>
         </is>
       </c>
     </row>
@@ -2702,12 +2846,12 @@
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>tooth-extraction page</t>
+          <t>wisdom-teeth-removal page</t>
         </is>
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/tustin-ca/tooth-extraction/</t>
+          <t>https://smiletustin.com/tustin-ca/wisdom-teeth-removal/</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
@@ -2737,12 +2881,12 @@
       </c>
       <c r="B61" s="7" t="inlineStr">
         <is>
-          <t>teeth-whitening page</t>
+          <t>teeth-cleaning page</t>
         </is>
       </c>
       <c r="C61" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/tustin-ca/teeth-whitening/</t>
+          <t>https://smiletustin.com/tustin-ca/teeth-cleaning/</t>
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr">
@@ -2760,7 +2904,7 @@
       <c r="H61" s="7" t="inlineStr"/>
       <c r="I61" s="7" t="inlineStr">
         <is>
-          <t>Best result for "teeth whitening tustin" (#1). Do not touch.</t>
+          <t>Title and heading match the page topic; no change needed now. Keep.</t>
         </is>
       </c>
     </row>
@@ -2772,12 +2916,12 @@
       </c>
       <c r="B62" s="7" t="inlineStr">
         <is>
-          <t>dental-crowns page</t>
+          <t>all-on-4-dental-implants page</t>
         </is>
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/tustin-ca/dental-crowns/</t>
+          <t>https://smiletustin.com/tustin-ca/all-on-4-dental-implants/</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
@@ -2807,12 +2951,12 @@
       </c>
       <c r="B63" s="7" t="inlineStr">
         <is>
-          <t>microscopic-micro-surgeries page</t>
+          <t>oral-surgery page</t>
         </is>
       </c>
       <c r="C63" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/tustin-ca/microscopic-micro-surgeries/</t>
+          <t>https://smiletustin.com/tustin-ca/oral-surgery/</t>
         </is>
       </c>
       <c r="D63" s="7" t="inlineStr">
@@ -2842,12 +2986,12 @@
       </c>
       <c r="B64" s="7" t="inlineStr">
         <is>
-          <t>contact-us page</t>
+          <t>dentures-and-partial-dentures page</t>
         </is>
       </c>
       <c r="C64" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/contact-us/</t>
+          <t>https://smiletustin.com/tustin-ca/dentures-and-partial-dentures/</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
@@ -2865,7 +3009,7 @@
       <c r="H64" s="7" t="inlineStr"/>
       <c r="I64" s="7" t="inlineStr">
         <is>
-          <t>Title and heading match the page topic; no change needed now. Keep.</t>
+          <t>Best result for "dentures tustin" (#1). Do not touch.</t>
         </is>
       </c>
     </row>
@@ -2877,12 +3021,12 @@
       </c>
       <c r="B65" s="7" t="inlineStr">
         <is>
-          <t>dental-implants page</t>
+          <t>tooth-extraction page</t>
         </is>
       </c>
       <c r="C65" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/tustin-ca/dental-implants/</t>
+          <t>https://smiletustin.com/tustin-ca/tooth-extraction/</t>
         </is>
       </c>
       <c r="D65" s="7" t="inlineStr">
@@ -2900,7 +3044,7 @@
       <c r="H65" s="7" t="inlineStr"/>
       <c r="I65" s="7" t="inlineStr">
         <is>
-          <t>Main dental implants service page; title and H1 match. Keep.</t>
+          <t>Title and heading match the page topic; no change needed now. Keep.</t>
         </is>
       </c>
     </row>
@@ -2912,12 +3056,12 @@
       </c>
       <c r="B66" s="7" t="inlineStr">
         <is>
-          <t>root-canals page</t>
+          <t>teeth-whitening page</t>
         </is>
       </c>
       <c r="C66" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/tustin-ca/root-canals/</t>
+          <t>https://smiletustin.com/tustin-ca/teeth-whitening/</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
@@ -2935,7 +3079,7 @@
       <c r="H66" s="7" t="inlineStr"/>
       <c r="I66" s="7" t="inlineStr">
         <is>
-          <t>Root canal service page; title and H1 match. Keep.</t>
+          <t>Best result for "teeth whitening tustin" (#1). Do not touch.</t>
         </is>
       </c>
     </row>
@@ -2947,12 +3091,12 @@
       </c>
       <c r="B67" s="7" t="inlineStr">
         <is>
-          <t>invisalign-clear-aligners page</t>
+          <t>dental-crowns page</t>
         </is>
       </c>
       <c r="C67" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/tustin-ca/invisalign-clear-aligners/</t>
+          <t>https://smiletustin.com/tustin-ca/dental-crowns/</t>
         </is>
       </c>
       <c r="D67" s="7" t="inlineStr">
@@ -2970,7 +3114,7 @@
       <c r="H67" s="7" t="inlineStr"/>
       <c r="I67" s="7" t="inlineStr">
         <is>
-          <t>Invisalign service page; title and H1 match. Keep.</t>
+          <t>Title and heading match the page topic; no change needed now. Keep.</t>
         </is>
       </c>
     </row>
@@ -2982,12 +3126,12 @@
       </c>
       <c r="B68" s="7" t="inlineStr">
         <is>
-          <t>laser-treatments page</t>
+          <t>microscopic-micro-surgeries page</t>
         </is>
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/tustin-ca/laser-treatments/</t>
+          <t>https://smiletustin.com/tustin-ca/microscopic-micro-surgeries/</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
@@ -3017,12 +3161,12 @@
       </c>
       <c r="B69" s="7" t="inlineStr">
         <is>
-          <t>how-does-light-therapy-speed-up-healing-after-dental-treatment page</t>
+          <t>contact-us page</t>
         </is>
       </c>
       <c r="C69" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/how-does-light-therapy-speed-up-healing-after-dental-treatment/</t>
+          <t>https://smiletustin.com/contact-us/</t>
         </is>
       </c>
       <c r="D69" s="7" t="inlineStr">
@@ -3040,7 +3184,7 @@
       <c r="H69" s="7" t="inlineStr"/>
       <c r="I69" s="7" t="inlineStr">
         <is>
-          <t>Blog article - title matches the topic and heading; on-topic. Keep.</t>
+          <t>Title and heading match the page topic; no change needed now. Keep.</t>
         </is>
       </c>
     </row>
@@ -3052,12 +3196,12 @@
       </c>
       <c r="B70" s="7" t="inlineStr">
         <is>
-          <t>can-untreated-tmj-damage-my-teeth-jaw-or-bite-long-term page</t>
+          <t>dental-implants page</t>
         </is>
       </c>
       <c r="C70" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/can-untreated-tmj-damage-my-teeth-jaw-or-bite-long-term/</t>
+          <t>https://smiletustin.com/tustin-ca/dental-implants/</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
@@ -3075,7 +3219,7 @@
       <c r="H70" s="7" t="inlineStr"/>
       <c r="I70" s="7" t="inlineStr">
         <is>
-          <t>Blog article - title matches the topic and heading; on-topic. Keep.</t>
+          <t>Main dental implants service page; title and H1 match. Keep.</t>
         </is>
       </c>
     </row>
@@ -3087,12 +3231,12 @@
       </c>
       <c r="B71" s="7" t="inlineStr">
         <is>
-          <t>what-should-i-do-if-my-aligner-tray-cracks-mid-treatment page</t>
+          <t>laser-treatments page</t>
         </is>
       </c>
       <c r="C71" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/what-should-i-do-if-my-aligner-tray-cracks-mid-treatment/</t>
+          <t>https://smiletustin.com/tustin-ca/laser-treatments/</t>
         </is>
       </c>
       <c r="D71" s="7" t="inlineStr">
@@ -3110,7 +3254,7 @@
       <c r="H71" s="7" t="inlineStr"/>
       <c r="I71" s="7" t="inlineStr">
         <is>
-          <t>Blog article - title matches the topic and heading; on-topic. Keep.</t>
+          <t>Title and heading match the page topic; no change needed now. Keep.</t>
         </is>
       </c>
     </row>
@@ -3122,12 +3266,12 @@
       </c>
       <c r="B72" s="7" t="inlineStr">
         <is>
-          <t>are-root-canals-painful-the-truth-from-smile-tustin page</t>
+          <t>how-does-light-therapy-speed-up-healing-after-dental-treatment page</t>
         </is>
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/are-root-canals-painful-the-truth-from-smile-tustin/</t>
+          <t>https://smiletustin.com/how-does-light-therapy-speed-up-healing-after-dental-treatment/</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
@@ -3145,7 +3289,7 @@
       <c r="H72" s="7" t="inlineStr"/>
       <c r="I72" s="7" t="inlineStr">
         <is>
-          <t>Blog that ranks and gets traffic; on-topic. Keep.</t>
+          <t>Blog article - title matches the topic and heading; on-topic. Keep.</t>
         </is>
       </c>
     </row>
@@ -3157,12 +3301,12 @@
       </c>
       <c r="B73" s="7" t="inlineStr">
         <is>
-          <t>can-laser-dentistry-fix-a-gummy-smile page</t>
+          <t>can-untreated-tmj-damage-my-teeth-jaw-or-bite-long-term page</t>
         </is>
       </c>
       <c r="C73" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/can-laser-dentistry-fix-a-gummy-smile/</t>
+          <t>https://smiletustin.com/can-untreated-tmj-damage-my-teeth-jaw-or-bite-long-term/</t>
         </is>
       </c>
       <c r="D73" s="7" t="inlineStr">
@@ -3192,12 +3336,12 @@
       </c>
       <c r="B74" s="7" t="inlineStr">
         <is>
-          <t>how-common-is-dental-implant-failure-and-what-causes-it-to-happen page</t>
+          <t>what-should-i-do-if-my-aligner-tray-cracks-mid-treatment page</t>
         </is>
       </c>
       <c r="C74" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/how-common-is-dental-implant-failure-and-what-causes-it-to-happen/</t>
+          <t>https://smiletustin.com/what-should-i-do-if-my-aligner-tray-cracks-mid-treatment/</t>
         </is>
       </c>
       <c r="D74" s="7" t="inlineStr">
@@ -3227,12 +3371,12 @@
       </c>
       <c r="B75" s="7" t="inlineStr">
         <is>
-          <t>dental-implants-and-diabetes-what-patients-need-to-know page</t>
+          <t>can-laser-dentistry-fix-a-gummy-smile page</t>
         </is>
       </c>
       <c r="C75" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/dental-implants-and-diabetes-what-patients-need-to-know/</t>
+          <t>https://smiletustin.com/can-laser-dentistry-fix-a-gummy-smile/</t>
         </is>
       </c>
       <c r="D75" s="7" t="inlineStr">
@@ -3262,12 +3406,12 @@
       </c>
       <c r="B76" s="7" t="inlineStr">
         <is>
-          <t>can-i-get-dental-implants-if-i-have-bone-loss page</t>
+          <t>how-common-is-dental-implant-failure-and-what-causes-it-to-happen page</t>
         </is>
       </c>
       <c r="C76" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/can-i-get-dental-implants-if-i-have-bone-loss/</t>
+          <t>https://smiletustin.com/how-common-is-dental-implant-failure-and-what-causes-it-to-happen/</t>
         </is>
       </c>
       <c r="D76" s="7" t="inlineStr">
@@ -3297,12 +3441,12 @@
       </c>
       <c r="B77" s="7" t="inlineStr">
         <is>
-          <t>our-tustin-dentist-explains-how-to-avoid-tooth-implant-complications page</t>
+          <t>dental-implants-and-diabetes-what-patients-need-to-know page</t>
         </is>
       </c>
       <c r="C77" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/our-tustin-dentist-explains-how-to-avoid-tooth-implant-complications/</t>
+          <t>https://smiletustin.com/dental-implants-and-diabetes-what-patients-need-to-know/</t>
         </is>
       </c>
       <c r="D77" s="7" t="inlineStr">
@@ -3332,12 +3476,12 @@
       </c>
       <c r="B78" s="7" t="inlineStr">
         <is>
-          <t>dental-implants-for-seniors-smile-tustin page</t>
+          <t>can-i-get-dental-implants-if-i-have-bone-loss page</t>
         </is>
       </c>
       <c r="C78" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/dental-implants-for-seniors-smile-tustin/</t>
+          <t>https://smiletustin.com/can-i-get-dental-implants-if-i-have-bone-loss/</t>
         </is>
       </c>
       <c r="D78" s="7" t="inlineStr">
@@ -3367,12 +3511,12 @@
       </c>
       <c r="B79" s="7" t="inlineStr">
         <is>
-          <t>emergency-tooth-implant-complications page</t>
+          <t>our-tustin-dentist-explains-how-to-avoid-tooth-implant-complications page</t>
         </is>
       </c>
       <c r="C79" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/emergency-tooth-implant-complications/</t>
+          <t>https://smiletustin.com/our-tustin-dentist-explains-how-to-avoid-tooth-implant-complications/</t>
         </is>
       </c>
       <c r="D79" s="7" t="inlineStr">
@@ -3402,12 +3546,12 @@
       </c>
       <c r="B80" s="7" t="inlineStr">
         <is>
-          <t>are-dental-implants-painful-to-get-at-smile-tustin page</t>
+          <t>dental-implants-for-seniors-smile-tustin page</t>
         </is>
       </c>
       <c r="C80" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/are-dental-implants-painful-to-get-at-smile-tustin/</t>
+          <t>https://smiletustin.com/dental-implants-for-seniors-smile-tustin/</t>
         </is>
       </c>
       <c r="D80" s="7" t="inlineStr">
@@ -3437,12 +3581,12 @@
       </c>
       <c r="B81" s="7" t="inlineStr">
         <is>
-          <t>are-implant-supported-dentures-right-for-you page</t>
+          <t>emergency-tooth-implant-complications page</t>
         </is>
       </c>
       <c r="C81" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/are-implant-supported-dentures-right-for-you/</t>
+          <t>https://smiletustin.com/emergency-tooth-implant-complications/</t>
         </is>
       </c>
       <c r="D81" s="7" t="inlineStr">
@@ -3472,12 +3616,12 @@
       </c>
       <c r="B82" s="7" t="inlineStr">
         <is>
-          <t>full-mouth-rehabilitation-smile-tustins-life-changing-prosthetic-solutions-for-complex-cases page</t>
+          <t>are-dental-implants-painful-to-get-at-smile-tustin page</t>
         </is>
       </c>
       <c r="C82" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/full-mouth-rehabilitation-smile-tustins-life-changing-prosthetic-solutions-for-complex-cases/</t>
+          <t>https://smiletustin.com/are-dental-implants-painful-to-get-at-smile-tustin/</t>
         </is>
       </c>
       <c r="D82" s="7" t="inlineStr">
@@ -3507,12 +3651,12 @@
       </c>
       <c r="B83" s="7" t="inlineStr">
         <is>
-          <t>dental-implants-are-they-worth-the-investment page</t>
+          <t>are-implant-supported-dentures-right-for-you page</t>
         </is>
       </c>
       <c r="C83" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/dental-implants-are-they-worth-the-investment/</t>
+          <t>https://smiletustin.com/are-implant-supported-dentures-right-for-you/</t>
         </is>
       </c>
       <c r="D83" s="7" t="inlineStr">
@@ -3542,12 +3686,12 @@
       </c>
       <c r="B84" s="7" t="inlineStr">
         <is>
-          <t>dental-implants-vs-bridges page</t>
+          <t>full-mouth-rehabilitation-smile-tustins-life-changing-prosthetic-solutions-for-complex-cases page</t>
         </is>
       </c>
       <c r="C84" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/dental-implants-vs-bridges/</t>
+          <t>https://smiletustin.com/full-mouth-rehabilitation-smile-tustins-life-changing-prosthetic-solutions-for-complex-cases/</t>
         </is>
       </c>
       <c r="D84" s="7" t="inlineStr">
@@ -3577,12 +3721,12 @@
       </c>
       <c r="B85" s="7" t="inlineStr">
         <is>
-          <t>smile-confidently-with-dental-implants page</t>
+          <t>dental-implants-are-they-worth-the-investment page</t>
         </is>
       </c>
       <c r="C85" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/smile-confidently-with-dental-implants/</t>
+          <t>https://smiletustin.com/dental-implants-are-they-worth-the-investment/</t>
         </is>
       </c>
       <c r="D85" s="7" t="inlineStr">
@@ -3612,12 +3756,12 @@
       </c>
       <c r="B86" s="7" t="inlineStr">
         <is>
-          <t>choosing-the-right-dental-implant-specialist-in-tustin-ca page</t>
+          <t>dental-implants-vs-bridges page</t>
         </is>
       </c>
       <c r="C86" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/choosing-the-right-dental-implant-specialist-in-tustin-ca/</t>
+          <t>https://smiletustin.com/dental-implants-vs-bridges/</t>
         </is>
       </c>
       <c r="D86" s="7" t="inlineStr">
@@ -3647,12 +3791,12 @@
       </c>
       <c r="B87" s="7" t="inlineStr">
         <is>
-          <t>am-i-a-candidate-for-dental-implants-in-tustin-ca page</t>
+          <t>smile-confidently-with-dental-implants page</t>
         </is>
       </c>
       <c r="C87" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/am-i-a-candidate-for-dental-implants-in-tustin-ca/</t>
+          <t>https://smiletustin.com/smile-confidently-with-dental-implants/</t>
         </is>
       </c>
       <c r="D87" s="7" t="inlineStr">
@@ -3682,12 +3826,12 @@
       </c>
       <c r="B88" s="7" t="inlineStr">
         <is>
-          <t>can-a-root-canal-procedure-save-your-tooth-in-tustin page</t>
+          <t>choosing-the-right-dental-implant-specialist-in-tustin-ca page</t>
         </is>
       </c>
       <c r="C88" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/can-a-root-canal-procedure-save-your-tooth-in-tustin/</t>
+          <t>https://smiletustin.com/choosing-the-right-dental-implant-specialist-in-tustin-ca/</t>
         </is>
       </c>
       <c r="D88" s="7" t="inlineStr">
@@ -3717,12 +3861,12 @@
       </c>
       <c r="B89" s="7" t="inlineStr">
         <is>
-          <t>factors-affect-root-canal-lifespan page</t>
+          <t>am-i-a-candidate-for-dental-implants-in-tustin-ca page</t>
         </is>
       </c>
       <c r="C89" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/factors-affect-root-canal-lifespan/</t>
+          <t>https://smiletustin.com/am-i-a-candidate-for-dental-implants-in-tustin-ca/</t>
         </is>
       </c>
       <c r="D89" s="7" t="inlineStr">
@@ -3752,12 +3896,12 @@
       </c>
       <c r="B90" s="7" t="inlineStr">
         <is>
-          <t>dentist-for-emergency-root-canal page</t>
+          <t>how-to-handle-a-toothache-when-dentist-offices-are-closed page</t>
         </is>
       </c>
       <c r="C90" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/dentist-for-emergency-root-canal/</t>
+          <t>https://smiletustin.com/how-to-handle-a-toothache-when-dentist-offices-are-closed/</t>
         </is>
       </c>
       <c r="D90" s="7" t="inlineStr">
@@ -3787,12 +3931,12 @@
       </c>
       <c r="B91" s="7" t="inlineStr">
         <is>
-          <t>beyond-teeth-whitening-internal-bleaching-for-discolored-root-canal-teeth page</t>
+          <t>weekend-toothache-your-options-when-the-dentist-isnt-available page</t>
         </is>
       </c>
       <c r="C91" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/beyond-teeth-whitening-internal-bleaching-for-discolored-root-canal-teeth/</t>
+          <t>https://smiletustin.com/weekend-toothache-your-options-when-the-dentist-isnt-available/</t>
         </is>
       </c>
       <c r="D91" s="7" t="inlineStr">
@@ -3822,12 +3966,12 @@
       </c>
       <c r="B92" s="7" t="inlineStr">
         <is>
-          <t>inside-smile-tustins-advanced-microscope-endodontics page</t>
+          <t>when-should-you-actually-call-an-emergency-dentist-near-me-in-tustin page</t>
         </is>
       </c>
       <c r="C92" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/inside-smile-tustins-advanced-microscope-endodontics/</t>
+          <t>https://smiletustin.com/when-should-you-actually-call-an-emergency-dentist-near-me-in-tustin/</t>
         </is>
       </c>
       <c r="D92" s="7" t="inlineStr">
@@ -3857,12 +4001,12 @@
       </c>
       <c r="B93" s="7" t="inlineStr">
         <is>
-          <t>the-truth-about-root-canals-why-theyre-not-what-you-think page</t>
+          <t>tooth-abscess-and-dental-emergencies-when-to-seek-immediate-care page</t>
         </is>
       </c>
       <c r="C93" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/the-truth-about-root-canals-why-theyre-not-what-you-think/</t>
+          <t>https://smiletustin.com/tooth-abscess-and-dental-emergencies-when-to-seek-immediate-care/</t>
         </is>
       </c>
       <c r="D93" s="7" t="inlineStr">
@@ -3880,7 +4024,7 @@
       <c r="H93" s="7" t="inlineStr"/>
       <c r="I93" s="7" t="inlineStr">
         <is>
-          <t>Root-canal blog that ranks and gets traffic; on-topic. Keep.</t>
+          <t>Blog article - title matches the topic and heading; on-topic. Keep.</t>
         </is>
       </c>
     </row>
@@ -3892,12 +4036,12 @@
       </c>
       <c r="B94" s="7" t="inlineStr">
         <is>
-          <t>am-i-a-candidate-for-root-canal-treatment-in-tustin-ca page</t>
+          <t>a-dentist-gives-tips-to-prevent-common-causes-of-toothaches page</t>
         </is>
       </c>
       <c r="C94" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/am-i-a-candidate-for-root-canal-treatment-in-tustin-ca/</t>
+          <t>https://smiletustin.com/a-dentist-gives-tips-to-prevent-common-causes-of-toothaches/</t>
         </is>
       </c>
       <c r="D94" s="7" t="inlineStr">
@@ -3927,12 +4071,12 @@
       </c>
       <c r="B95" s="7" t="inlineStr">
         <is>
-          <t>how-to-handle-a-toothache-when-dentist-offices-are-closed page</t>
+          <t>invisalign-vs-braces-which-option-works-better-for-younger-patients page</t>
         </is>
       </c>
       <c r="C95" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/how-to-handle-a-toothache-when-dentist-offices-are-closed/</t>
+          <t>https://smiletustin.com/invisalign-vs-braces-which-option-works-better-for-younger-patients/</t>
         </is>
       </c>
       <c r="D95" s="7" t="inlineStr">
@@ -3962,12 +4106,12 @@
       </c>
       <c r="B96" s="7" t="inlineStr">
         <is>
-          <t>weekend-toothache-your-options-when-the-dentist-isnt-available page</t>
+          <t>bothered-by-teeth-that-flare-out-heres-how-to-fix-them page</t>
         </is>
       </c>
       <c r="C96" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/weekend-toothache-your-options-when-the-dentist-isnt-available/</t>
+          <t>https://smiletustin.com/bothered-by-teeth-that-flare-out-heres-how-to-fix-them/</t>
         </is>
       </c>
       <c r="D96" s="7" t="inlineStr">
@@ -3997,12 +4141,12 @@
       </c>
       <c r="B97" s="7" t="inlineStr">
         <is>
-          <t>when-should-you-actually-call-an-emergency-dentist-near-me-in-tustin page</t>
+          <t>invisalign-clear-aligners-why-retainers-matter-more-than-you-think page</t>
         </is>
       </c>
       <c r="C97" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/when-should-you-actually-call-an-emergency-dentist-near-me-in-tustin/</t>
+          <t>https://smiletustin.com/invisalign-clear-aligners-why-retainers-matter-more-than-you-think/</t>
         </is>
       </c>
       <c r="D97" s="7" t="inlineStr">
@@ -4032,12 +4176,12 @@
       </c>
       <c r="B98" s="7" t="inlineStr">
         <is>
-          <t>emergency-dental-care-in-tustin-where-to-go-when-tooth-pain-strikes page</t>
+          <t>lost-invisalign-aligners-in-tustin page</t>
         </is>
       </c>
       <c r="C98" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/emergency-dental-care-in-tustin-where-to-go-when-tooth-pain-strikes/</t>
+          <t>https://smiletustin.com/lost-invisalign-aligners-in-tustin/</t>
         </is>
       </c>
       <c r="D98" s="7" t="inlineStr">
@@ -4067,12 +4211,12 @@
       </c>
       <c r="B99" s="7" t="inlineStr">
         <is>
-          <t>tooth-abscess-and-dental-emergencies-when-to-seek-immediate-care page</t>
+          <t>invisalign-for-teens-builds-confidence page</t>
         </is>
       </c>
       <c r="C99" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/tooth-abscess-and-dental-emergencies-when-to-seek-immediate-care/</t>
+          <t>https://smiletustin.com/invisalign-for-teens-builds-confidence/</t>
         </is>
       </c>
       <c r="D99" s="7" t="inlineStr">
@@ -4102,12 +4246,12 @@
       </c>
       <c r="B100" s="7" t="inlineStr">
         <is>
-          <t>a-dentist-gives-tips-to-prevent-common-causes-of-toothaches page</t>
+          <t>caring-for-invisalign-aligners-during-the-holidays page</t>
         </is>
       </c>
       <c r="C100" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/a-dentist-gives-tips-to-prevent-common-causes-of-toothaches/</t>
+          <t>https://smiletustin.com/caring-for-invisalign-aligners-during-the-holidays/</t>
         </is>
       </c>
       <c r="D100" s="7" t="inlineStr">
@@ -4137,12 +4281,12 @@
       </c>
       <c r="B101" s="7" t="inlineStr">
         <is>
-          <t>invisalign-vs-braces-which-option-works-better-for-younger-patients page</t>
+          <t>how-can-a-dentist-fix-a-gap-between-front-teeth page</t>
         </is>
       </c>
       <c r="C101" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/invisalign-vs-braces-which-option-works-better-for-younger-patients/</t>
+          <t>https://smiletustin.com/how-can-a-dentist-fix-a-gap-between-front-teeth/</t>
         </is>
       </c>
       <c r="D101" s="7" t="inlineStr">
@@ -4160,7 +4304,7 @@
       <c r="H101" s="7" t="inlineStr"/>
       <c r="I101" s="7" t="inlineStr">
         <is>
-          <t>Blog article - title matches the topic and heading; on-topic. Keep.</t>
+          <t>Blog that ranks and gets traffic; on-topic. Keep.</t>
         </is>
       </c>
     </row>
@@ -4172,12 +4316,12 @@
       </c>
       <c r="B102" s="7" t="inlineStr">
         <is>
-          <t>bothered-by-teeth-that-flare-out-heres-how-to-fix-them page</t>
+          <t>cosmetic-treatments-how-we-create-smile-makeovers-in-tustin page</t>
         </is>
       </c>
       <c r="C102" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/bothered-by-teeth-that-flare-out-heres-how-to-fix-them/</t>
+          <t>https://smiletustin.com/cosmetic-treatments-how-we-create-smile-makeovers-in-tustin/</t>
         </is>
       </c>
       <c r="D102" s="7" t="inlineStr">
@@ -4207,12 +4351,12 @@
       </c>
       <c r="B103" s="7" t="inlineStr">
         <is>
-          <t>invisalign-clear-aligners-why-retainers-matter-more-than-you-think page</t>
+          <t>top-5-tips-for-caring-for-tustin-cosmetic-teeth-veneers page</t>
         </is>
       </c>
       <c r="C103" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/invisalign-clear-aligners-why-retainers-matter-more-than-you-think/</t>
+          <t>https://smiletustin.com/top-5-tips-for-caring-for-tustin-cosmetic-teeth-veneers/</t>
         </is>
       </c>
       <c r="D103" s="7" t="inlineStr">
@@ -4242,12 +4386,12 @@
       </c>
       <c r="B104" s="7" t="inlineStr">
         <is>
-          <t>lost-invisalign-aligners-in-tustin page</t>
+          <t>cosmetic-dentistry-tustin-achieve-your-best-smile page</t>
         </is>
       </c>
       <c r="C104" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/lost-invisalign-aligners-in-tustin/</t>
+          <t>https://smiletustin.com/cosmetic-dentistry-tustin-achieve-your-best-smile/</t>
         </is>
       </c>
       <c r="D104" s="7" t="inlineStr">
@@ -4277,12 +4421,12 @@
       </c>
       <c r="B105" s="7" t="inlineStr">
         <is>
-          <t>invisalign-for-teens-builds-confidence page</t>
+          <t>what-are-the-early-signs-of-oral-cancer-that-most-people-miss page</t>
         </is>
       </c>
       <c r="C105" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/invisalign-for-teens-builds-confidence/</t>
+          <t>https://smiletustin.com/what-are-the-early-signs-of-oral-cancer-that-most-people-miss/</t>
         </is>
       </c>
       <c r="D105" s="7" t="inlineStr">
@@ -4312,12 +4456,12 @@
       </c>
       <c r="B106" s="7" t="inlineStr">
         <is>
-          <t>caring-for-invisalign-aligners-during-the-holidays page</t>
+          <t>what-is-the-white-stuff-on-your-teeth-even-after-you-brush page</t>
         </is>
       </c>
       <c r="C106" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/caring-for-invisalign-aligners-during-the-holidays/</t>
+          <t>https://smiletustin.com/what-is-the-white-stuff-on-your-teeth-even-after-you-brush/</t>
         </is>
       </c>
       <c r="D106" s="7" t="inlineStr">
@@ -4335,7 +4479,7 @@
       <c r="H106" s="7" t="inlineStr"/>
       <c r="I106" s="7" t="inlineStr">
         <is>
-          <t>Blog article - title matches the topic and heading; on-topic. Keep.</t>
+          <t>Blog that ranks and gets traffic; on-topic. Keep.</t>
         </is>
       </c>
     </row>
@@ -4347,12 +4491,12 @@
       </c>
       <c r="B107" s="7" t="inlineStr">
         <is>
-          <t>how-can-a-dentist-fix-a-gap-between-front-teeth page</t>
+          <t>how-prp-and-prf-therapy-accelerates-your-dental-recovery-in-tustin page</t>
         </is>
       </c>
       <c r="C107" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/how-can-a-dentist-fix-a-gap-between-front-teeth/</t>
+          <t>https://smiletustin.com/how-prp-and-prf-therapy-accelerates-your-dental-recovery-in-tustin/</t>
         </is>
       </c>
       <c r="D107" s="7" t="inlineStr">
@@ -4370,7 +4514,7 @@
       <c r="H107" s="7" t="inlineStr"/>
       <c r="I107" s="7" t="inlineStr">
         <is>
-          <t>Blog that ranks and gets traffic; on-topic. Keep.</t>
+          <t>Blog article - title matches the topic and heading; on-topic. Keep.</t>
         </is>
       </c>
     </row>
@@ -4382,12 +4526,12 @@
       </c>
       <c r="B108" s="7" t="inlineStr">
         <is>
-          <t>cosmetic-treatments-how-we-create-smile-makeovers-in-tustin page</t>
+          <t>precision-dentistry-the-art-of-microscopic-microsurgeries-at-smile-tustin page</t>
         </is>
       </c>
       <c r="C108" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/cosmetic-treatments-how-we-create-smile-makeovers-in-tustin/</t>
+          <t>https://smiletustin.com/precision-dentistry-the-art-of-microscopic-microsurgeries-at-smile-tustin/</t>
         </is>
       </c>
       <c r="D108" s="7" t="inlineStr">
@@ -4417,12 +4561,12 @@
       </c>
       <c r="B109" s="7" t="inlineStr">
         <is>
-          <t>top-5-tips-for-caring-for-tustin-cosmetic-teeth-veneers page</t>
+          <t>jaw-pain-relief-smile-tustins-tmj-therapy-changing-lives-in-tustin-and-beyond page</t>
         </is>
       </c>
       <c r="C109" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/top-5-tips-for-caring-for-tustin-cosmetic-teeth-veneers/</t>
+          <t>https://smiletustin.com/jaw-pain-relief-smile-tustins-tmj-therapy-changing-lives-in-tustin-and-beyond/</t>
         </is>
       </c>
       <c r="D109" s="7" t="inlineStr">
@@ -4452,12 +4596,12 @@
       </c>
       <c r="B110" s="7" t="inlineStr">
         <is>
-          <t>cosmetic-dentistry-tustin-achieve-your-best-smile page</t>
+          <t>dental-implants-cost-guide-tustin-ca page</t>
         </is>
       </c>
       <c r="C110" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/cosmetic-dentistry-tustin-achieve-your-best-smile/</t>
+          <t>https://smiletustin.com/dental-implants-cost-guide-tustin-ca/</t>
         </is>
       </c>
       <c r="D110" s="7" t="inlineStr">
@@ -4475,7 +4619,7 @@
       <c r="H110" s="7" t="inlineStr"/>
       <c r="I110" s="7" t="inlineStr">
         <is>
-          <t>Blog article - title matches the topic and heading; on-topic. Keep.</t>
+          <t>Top implant blog (page 1 for several "dental implants tustin" terms) and the biggest traffic driver after the home page. Do not touch.</t>
         </is>
       </c>
     </row>
@@ -4487,12 +4631,12 @@
       </c>
       <c r="B111" s="7" t="inlineStr">
         <is>
-          <t>what-are-the-early-signs-of-oral-cancer-that-most-people-miss page</t>
+          <t>do-i-have-sleep-apnea-or-am-i-just-a-loud-snorer page</t>
         </is>
       </c>
       <c r="C111" s="7" t="inlineStr">
         <is>
-          <t>https://smiletustin.com/what-are-the-early-signs-of-oral-cancer-that-most-people-miss/</t>
+          <t>https://smiletustin.com/do-i-have-sleep-apnea-or-am-i-just-a-loud-snorer/</t>
         </is>
       </c>
       <c r="D111" s="7" t="inlineStr">
@@ -4514,288 +4658,8 @@
         </is>
       </c>
     </row>
-    <row r="112">
-      <c r="A112" s="7" t="inlineStr">
-        <is>
-          <t>111</t>
-        </is>
-      </c>
-      <c r="B112" s="7" t="inlineStr">
-        <is>
-          <t>what-is-the-white-stuff-on-your-teeth-even-after-you-brush page</t>
-        </is>
-      </c>
-      <c r="C112" s="7" t="inlineStr">
-        <is>
-          <t>https://smiletustin.com/what-is-the-white-stuff-on-your-teeth-even-after-you-brush/</t>
-        </is>
-      </c>
-      <c r="D112" s="7" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="E112" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F112" s="7" t="inlineStr"/>
-      <c r="G112" s="7" t="inlineStr"/>
-      <c r="H112" s="7" t="inlineStr"/>
-      <c r="I112" s="7" t="inlineStr">
-        <is>
-          <t>Blog that ranks and gets traffic; on-topic. Keep.</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" s="7" t="inlineStr">
-        <is>
-          <t>112</t>
-        </is>
-      </c>
-      <c r="B113" s="7" t="inlineStr">
-        <is>
-          <t>tustin-teeth-cleaning-appointment page</t>
-        </is>
-      </c>
-      <c r="C113" s="7" t="inlineStr">
-        <is>
-          <t>https://smiletustin.com/tustin-teeth-cleaning-appointment/</t>
-        </is>
-      </c>
-      <c r="D113" s="7" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="E113" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F113" s="7" t="inlineStr"/>
-      <c r="G113" s="7" t="inlineStr"/>
-      <c r="H113" s="7" t="inlineStr"/>
-      <c r="I113" s="7" t="inlineStr">
-        <is>
-          <t>Blog article - title matches the topic and heading; on-topic. Keep.</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" s="7" t="inlineStr">
-        <is>
-          <t>113</t>
-        </is>
-      </c>
-      <c r="B114" s="7" t="inlineStr">
-        <is>
-          <t>how-prp-and-prf-therapy-accelerates-your-dental-recovery-in-tustin page</t>
-        </is>
-      </c>
-      <c r="C114" s="7" t="inlineStr">
-        <is>
-          <t>https://smiletustin.com/how-prp-and-prf-therapy-accelerates-your-dental-recovery-in-tustin/</t>
-        </is>
-      </c>
-      <c r="D114" s="7" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="E114" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F114" s="7" t="inlineStr"/>
-      <c r="G114" s="7" t="inlineStr"/>
-      <c r="H114" s="7" t="inlineStr"/>
-      <c r="I114" s="7" t="inlineStr">
-        <is>
-          <t>Blog article - title matches the topic and heading; on-topic. Keep.</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" s="7" t="inlineStr">
-        <is>
-          <t>114</t>
-        </is>
-      </c>
-      <c r="B115" s="7" t="inlineStr">
-        <is>
-          <t>precision-dentistry-the-art-of-microscopic-microsurgeries-at-smile-tustin page</t>
-        </is>
-      </c>
-      <c r="C115" s="7" t="inlineStr">
-        <is>
-          <t>https://smiletustin.com/precision-dentistry-the-art-of-microscopic-microsurgeries-at-smile-tustin/</t>
-        </is>
-      </c>
-      <c r="D115" s="7" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="E115" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F115" s="7" t="inlineStr"/>
-      <c r="G115" s="7" t="inlineStr"/>
-      <c r="H115" s="7" t="inlineStr"/>
-      <c r="I115" s="7" t="inlineStr">
-        <is>
-          <t>Blog article - title matches the topic and heading; on-topic. Keep.</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" s="7" t="inlineStr">
-        <is>
-          <t>115</t>
-        </is>
-      </c>
-      <c r="B116" s="7" t="inlineStr">
-        <is>
-          <t>jaw-pain-relief-smile-tustins-tmj-therapy-changing-lives-in-tustin-and-beyond page</t>
-        </is>
-      </c>
-      <c r="C116" s="7" t="inlineStr">
-        <is>
-          <t>https://smiletustin.com/jaw-pain-relief-smile-tustins-tmj-therapy-changing-lives-in-tustin-and-beyond/</t>
-        </is>
-      </c>
-      <c r="D116" s="7" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="E116" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F116" s="7" t="inlineStr"/>
-      <c r="G116" s="7" t="inlineStr"/>
-      <c r="H116" s="7" t="inlineStr"/>
-      <c r="I116" s="7" t="inlineStr">
-        <is>
-          <t>Blog article - title matches the topic and heading; on-topic. Keep.</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" s="7" t="inlineStr">
-        <is>
-          <t>116</t>
-        </is>
-      </c>
-      <c r="B117" s="7" t="inlineStr">
-        <is>
-          <t>new-year-new-smile-find-your-local-dentist-in-tustin-for-2026 page</t>
-        </is>
-      </c>
-      <c r="C117" s="7" t="inlineStr">
-        <is>
-          <t>https://smiletustin.com/new-year-new-smile-find-your-local-dentist-in-tustin-for-2026/</t>
-        </is>
-      </c>
-      <c r="D117" s="7" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="E117" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F117" s="7" t="inlineStr"/>
-      <c r="G117" s="7" t="inlineStr"/>
-      <c r="H117" s="7" t="inlineStr"/>
-      <c r="I117" s="7" t="inlineStr">
-        <is>
-          <t>Blog article - title matches the topic and heading; on-topic. Keep.</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="7" t="inlineStr">
-        <is>
-          <t>117</t>
-        </is>
-      </c>
-      <c r="B118" s="7" t="inlineStr">
-        <is>
-          <t>dental-implants-cost-guide-tustin-ca page</t>
-        </is>
-      </c>
-      <c r="C118" s="7" t="inlineStr">
-        <is>
-          <t>https://smiletustin.com/dental-implants-cost-guide-tustin-ca/</t>
-        </is>
-      </c>
-      <c r="D118" s="7" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="E118" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F118" s="7" t="inlineStr"/>
-      <c r="G118" s="7" t="inlineStr"/>
-      <c r="H118" s="7" t="inlineStr"/>
-      <c r="I118" s="7" t="inlineStr">
-        <is>
-          <t>Top implant blog (page 1 for several "dental implants tustin" terms) and the biggest traffic driver after the home page. Do not touch.</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" s="7" t="inlineStr">
-        <is>
-          <t>118</t>
-        </is>
-      </c>
-      <c r="B119" s="7" t="inlineStr">
-        <is>
-          <t>do-i-have-sleep-apnea-or-am-i-just-a-loud-snorer page</t>
-        </is>
-      </c>
-      <c r="C119" s="7" t="inlineStr">
-        <is>
-          <t>https://smiletustin.com/do-i-have-sleep-apnea-or-am-i-just-a-loud-snorer/</t>
-        </is>
-      </c>
-      <c r="D119" s="7" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="E119" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F119" s="7" t="inlineStr"/>
-      <c r="G119" s="7" t="inlineStr"/>
-      <c r="H119" s="7" t="inlineStr"/>
-      <c r="I119" s="7" t="inlineStr">
-        <is>
-          <t>Blog article - title matches the topic and heading; on-topic. Keep.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:I119"/>
+  <autoFilter ref="A1:I111"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>